<commit_message>
Restate AdTech summary on one logic; master v4: CONS revenue w/o ADJ + report archive
- Master_AT_Sep_v4: 15 CONS revenue = 12 Segments rows 13+15 (BiP increment w/o e-com, w/o ADJ);
  model block (rows 71-77) and value archive of reported months (rows 81-87, Jan-Aug filled);
  rows 6/7/39/40/53/57/59 take archive when filled; check row 67 compares the model block.
- Summary: Jan-Dec rebuilt from v4; sheet 'Было → стало' with old vs new.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142u1JgEJ5Z4iqbgjpLWfcB
</commit_message>
<xml_diff>
--- a/Adtech_svod_Aug-Sep_fact_Oct-Dec_FC.xlsx
+++ b/Adtech_svod_Aug-Sep_fact_Oct-Dec_FC.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Свод" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Было → стало" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -15,12 +16,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0;[Red]-#,##0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <charset val="204"/>
@@ -88,6 +90,9 @@
       <color rgb="FFFF0000"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -205,7 +210,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -321,6 +326,8 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="3"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -701,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:N64"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="51.83203125" customWidth="1" min="1" max="1"/>
@@ -709,6 +716,13 @@
     <col width="11.1640625" customWidth="1" style="35" min="14" max="14"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>сен — предв. факт (Rev до финальной сверки)</t>
+        </is>
+      </c>
+    </row>
     <row r="2" ht="16" customHeight="1" thickBot="1">
       <c r="B2" s="38" t="inlineStr">
         <is>
@@ -1086,40 +1100,40 @@
         </is>
       </c>
       <c r="B16" s="18" t="n">
-        <v>79925999.34437963</v>
+        <v>76370133.2853148</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>141070480.6976929</v>
+        <v>29324504.16163935</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>132973014.0892157</v>
+        <v>22506699.26600663</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>161307290.0874327</v>
+        <v>65792079.21795091</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>328261556.6602637</v>
+        <v>158474111.2911011</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>437761061.4028037</v>
+        <v>155081968.7122735</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>261366316.2682095</v>
+        <v>261366316.2682093</v>
       </c>
       <c r="I16" s="18" t="n">
         <v>253412062.0304224</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>434087500.8000364</v>
+        <v>434087500.8000365</v>
       </c>
       <c r="K16" s="18" t="n">
         <v>253547548.1809133</v>
       </c>
       <c r="L16" s="18" t="n">
-        <v>302722641.8468388</v>
+        <v>302722641.8468389</v>
       </c>
       <c r="M16" s="18" t="n">
-        <v>393067327.6715648</v>
+        <v>393067327.6715649</v>
       </c>
       <c r="N16" s="36" t="n"/>
     </row>
@@ -1310,40 +1324,40 @@
         </is>
       </c>
       <c r="B26" s="24" t="n">
-        <v>79925999.34437963</v>
+        <v>76370133.2853148</v>
       </c>
       <c r="C26" s="24" t="n">
-        <v>141070480.6976929</v>
+        <v>29324504.16163935</v>
       </c>
       <c r="D26" s="24" t="n">
-        <v>132973014.0892157</v>
+        <v>22506699.26600663</v>
       </c>
       <c r="E26" s="24" t="n">
-        <v>161307290.0874327</v>
+        <v>65792079.21795091</v>
       </c>
       <c r="F26" s="24" t="n">
-        <v>328261556.6602637</v>
+        <v>158474111.2911011</v>
       </c>
       <c r="G26" s="24" t="n">
-        <v>437761061.4028037</v>
+        <v>155081968.7122735</v>
       </c>
       <c r="H26" s="24" t="n">
-        <v>261366316.2682095</v>
+        <v>261366316.2682093</v>
       </c>
       <c r="I26" s="24" t="n">
         <v>253412062.0304224</v>
       </c>
       <c r="J26" s="24" t="n">
-        <v>434087500.8000364</v>
+        <v>434087500.8000365</v>
       </c>
       <c r="K26" s="24" t="n">
         <v>253547548.1809133</v>
       </c>
       <c r="L26" s="24" t="n">
-        <v>302722641.8468388</v>
+        <v>302722641.8468389</v>
       </c>
       <c r="M26" s="24" t="n">
-        <v>393067327.6715648</v>
+        <v>393067327.6715649</v>
       </c>
       <c r="N26" s="36" t="n"/>
     </row>
@@ -1414,25 +1428,25 @@
         </is>
       </c>
       <c r="B30" s="26" t="n">
-        <v>-125342678.15</v>
+        <v>-125338709.1217621</v>
       </c>
       <c r="C30" s="26" t="n">
-        <v>-99252146.21000001</v>
+        <v>-114315781.0228943</v>
       </c>
       <c r="D30" s="26" t="n">
-        <v>-86709865.21020025</v>
+        <v>-124304616.3602002</v>
       </c>
       <c r="E30" s="26" t="n">
-        <v>-193324661.3008188</v>
+        <v>-141645834.3208189</v>
       </c>
       <c r="F30" s="26" t="n">
-        <v>-160146548.3796875</v>
+        <v>-158979393.6550312</v>
       </c>
       <c r="G30" s="26" t="n">
-        <v>-243860194.9635304</v>
+        <v>-231411491.7358956</v>
       </c>
       <c r="H30" s="26" t="n">
-        <v>-224839257.3646601</v>
+        <v>-237266483.1622952</v>
       </c>
       <c r="I30" s="26" t="n">
         <v>-204575265.598262</v>
@@ -1478,25 +1492,25 @@
         </is>
       </c>
       <c r="B32" s="18" t="n">
-        <v>-95938090.5</v>
+        <v>-95889496.05176206</v>
       </c>
       <c r="C32" s="18" t="n">
-        <v>-95034802.90000001</v>
+        <v>-94986109.7028943</v>
       </c>
       <c r="D32" s="18" t="n">
-        <v>-96333821.15020025</v>
+        <v>-96303006.88020022</v>
       </c>
       <c r="E32" s="18" t="n">
-        <v>-103523767.9508188</v>
+        <v>-103490005.6108189</v>
       </c>
       <c r="F32" s="18" t="n">
-        <v>-113707319.5496875</v>
+        <v>-112891591.6250312</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>-122657190.2135303</v>
+        <v>-110994514.3958956</v>
       </c>
       <c r="H32" s="18" t="n">
-        <v>-99072375.46466005</v>
+        <v>-111712643.4622951</v>
       </c>
       <c r="I32" s="18" t="n">
         <v>-114474730.038262</v>
@@ -1562,25 +1576,25 @@
         </is>
       </c>
       <c r="B35" s="18" t="n">
-        <v>-92886360.5</v>
+        <v>-89794141.17176206</v>
       </c>
       <c r="C35" s="18" t="n">
-        <v>-94592513.90000001</v>
+        <v>-91055814.04346746</v>
       </c>
       <c r="D35" s="18" t="n">
-        <v>-95109178.44724879</v>
+        <v>-91790548.47724877</v>
       </c>
       <c r="E35" s="18" t="n">
-        <v>-101882236.5107256</v>
+        <v>-102521792.3807257</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>-112467620.9260646</v>
+        <v>-106126609.8708351</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>-106240266.7461649</v>
+        <v>-109249003.0885301</v>
       </c>
       <c r="H35" s="18" t="n">
-        <v>-101336835.3946933</v>
+        <v>-113977103.3923284</v>
       </c>
       <c r="I35" s="18" t="n">
         <v>-111304741.7725611</v>
@@ -1606,25 +1620,25 @@
         </is>
       </c>
       <c r="B36" s="22" t="n">
-        <v>-3051730</v>
+        <v>-6095354.88</v>
       </c>
       <c r="C36" s="22" t="n">
-        <v>-442289</v>
+        <v>-3930295.659426838</v>
       </c>
       <c r="D36" s="22" t="n">
-        <v>-1224642.702951454</v>
+        <v>-4512458.402951454</v>
       </c>
       <c r="E36" s="22" t="n">
-        <v>-1641531.440093187</v>
+        <v>-968213.2300931871</v>
       </c>
       <c r="F36" s="22" t="n">
-        <v>-1239698.623622975</v>
+        <v>-6764981.754196137</v>
       </c>
       <c r="G36" s="22" t="n">
-        <v>-16416923.46736547</v>
+        <v>-1745511.307365466</v>
       </c>
       <c r="H36" s="22" t="n">
-        <v>2264459.930033199</v>
+        <v>2264459.9300332</v>
       </c>
       <c r="I36" s="22" t="n">
         <v>-3169988.265700941</v>
@@ -1650,25 +1664,25 @@
         </is>
       </c>
       <c r="B37" s="30" t="n">
-        <v>-29404587.65</v>
+        <v>-29449213.07</v>
       </c>
       <c r="C37" s="30" t="n">
-        <v>-4217343.310000001</v>
+        <v>-19329671.32</v>
       </c>
       <c r="D37" s="30" t="n">
-        <v>9623955.939999999</v>
+        <v>-28001609.48</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>-89800893.35000001</v>
+        <v>-38155828.71000001</v>
       </c>
       <c r="F37" s="30" t="n">
-        <v>-46439228.82999997</v>
+        <v>-46087802.03</v>
       </c>
       <c r="G37" s="30" t="n">
-        <v>-121203004.75</v>
+        <v>-120416977.34</v>
       </c>
       <c r="H37" s="30" t="n">
-        <v>-125766881.9</v>
+        <v>-125553839.7</v>
       </c>
       <c r="I37" s="30" t="n">
         <v>-90100535.56</v>
@@ -1914,25 +1928,25 @@
         </is>
       </c>
       <c r="B49" s="18" t="n">
-        <v>-28528894</v>
+        <v>-28528894.09</v>
       </c>
       <c r="C49" s="18" t="n">
-        <v>-1745000</v>
+        <v>-16829134.28</v>
       </c>
       <c r="D49" s="18" t="n">
-        <v>9535203.629999999</v>
+        <v>-27059488.98</v>
       </c>
       <c r="E49" s="18" t="n">
-        <v>-87759899.82000002</v>
+        <v>-36081072.84000001</v>
       </c>
       <c r="F49" s="18" t="n">
-        <v>-43871683.96999997</v>
+        <v>-43768464.97</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>-106620550.19</v>
+        <v>-106723769.19</v>
       </c>
       <c r="H49" s="18" t="n">
-        <v>-120266758.59</v>
+        <v>-120265799.17</v>
       </c>
       <c r="I49" s="18" t="n">
         <v>-82797191.41</v>
@@ -2018,25 +2032,25 @@
         </is>
       </c>
       <c r="B53" s="19" t="n">
-        <v>-155854</v>
+        <v>-155853.97</v>
       </c>
       <c r="C53" s="19" t="n">
-        <v>-1633817</v>
+        <v>-1633816.65</v>
       </c>
       <c r="D53" s="19" t="n">
-        <v>772474.76</v>
+        <v>-203115.78</v>
       </c>
       <c r="E53" s="19" t="n">
         <v>-1371206.32</v>
       </c>
       <c r="F53" s="19" t="n">
-        <v>-2464153.540000001</v>
+        <v>-1488563.38</v>
       </c>
       <c r="G53" s="19" t="n">
-        <v>-2164074.739999998</v>
+        <v>-2164074.74</v>
       </c>
       <c r="H53" s="19" t="n">
-        <v>-940167.4499999998</v>
+        <v>-722153.7499999998</v>
       </c>
       <c r="I53" s="19" t="n">
         <v>-964293.23</v>
@@ -2082,25 +2096,25 @@
         </is>
       </c>
       <c r="B55" s="18" t="n">
-        <v>-719839.65</v>
+        <v>-764465.0100000001</v>
       </c>
       <c r="C55" s="18" t="n">
-        <v>-838526.3100000001</v>
+        <v>-866720.39</v>
       </c>
       <c r="D55" s="18" t="n">
-        <v>-683722.4500000001</v>
+        <v>-739004.72</v>
       </c>
       <c r="E55" s="18" t="n">
-        <v>-669787.2100000001</v>
+        <v>-703549.55</v>
       </c>
       <c r="F55" s="18" t="n">
-        <v>-103391.3200000003</v>
+        <v>-830773.6799999999</v>
       </c>
       <c r="G55" s="18" t="n">
-        <v>-12418379.82</v>
+        <v>-11529133.41</v>
       </c>
       <c r="H55" s="18" t="n">
-        <v>-4559955.859999999</v>
+        <v>-4565886.779999999</v>
       </c>
       <c r="I55" s="18" t="n">
         <v>-6339050.920000001</v>
@@ -2206,25 +2220,25 @@
         </is>
       </c>
       <c r="B60" s="24" t="n">
-        <v>-45416678.80562037</v>
+        <v>-48968575.83644727</v>
       </c>
       <c r="C60" s="24" t="n">
-        <v>41818334.48769292</v>
+        <v>-84991276.86125495</v>
       </c>
       <c r="D60" s="24" t="n">
-        <v>46263148.87901543</v>
+        <v>-101797917.0941936</v>
       </c>
       <c r="E60" s="24" t="n">
-        <v>-32017371.21338606</v>
+        <v>-75853755.10286799</v>
       </c>
       <c r="F60" s="24" t="n">
-        <v>168115008.2805762</v>
+        <v>-505282.3639300764</v>
       </c>
       <c r="G60" s="24" t="n">
-        <v>193900866.4392734</v>
+        <v>-76329523.02362204</v>
       </c>
       <c r="H60" s="24" t="n">
-        <v>36527058.90354943</v>
+        <v>24099833.10591418</v>
       </c>
       <c r="I60" s="24" t="n">
         <v>48836796.43216032</v>
@@ -2236,7 +2250,7 @@
         <v>26741437.57239074</v>
       </c>
       <c r="L60" s="24" t="n">
-        <v>81862498.51519418</v>
+        <v>81862498.51519424</v>
       </c>
       <c r="M60" s="24" t="n">
         <v>157385839.4906691</v>
@@ -2295,4 +2309,1870 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Сверка: прежний свод (v93) → новый свод (Master_AT_Sep_v4, единая логика), млн руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>Commercial margin</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B4" s="42" t="n">
+        <v>79.92599934437963</v>
+      </c>
+      <c r="C4" s="42" t="n">
+        <v>141.0704806976929</v>
+      </c>
+      <c r="D4" s="42" t="n">
+        <v>132.9730140892157</v>
+      </c>
+      <c r="E4" s="42" t="n">
+        <v>161.3072900874327</v>
+      </c>
+      <c r="F4" s="42" t="n">
+        <v>328.2615566602636</v>
+      </c>
+      <c r="G4" s="42" t="n">
+        <v>437.7610614028037</v>
+      </c>
+      <c r="H4" s="42" t="n">
+        <v>261.3663162682095</v>
+      </c>
+      <c r="I4" s="42" t="n">
+        <v>75.15798898306431</v>
+      </c>
+      <c r="J4" s="42" t="n">
+        <v>69.58021505923334</v>
+      </c>
+      <c r="K4" s="42" t="n">
+        <v>1.998088570723601</v>
+      </c>
+      <c r="L4" s="42" t="n">
+        <v>53.30722195520254</v>
+      </c>
+      <c r="M4" s="42" t="n">
+        <v>74.57192641253258</v>
+      </c>
+      <c r="N4" s="42" t="n">
+        <v>1542.665718549998</v>
+      </c>
+      <c r="O4" s="42" t="n">
+        <v>1817.281159530754</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B5" s="42" t="n">
+        <v>76.37013328531479</v>
+      </c>
+      <c r="C5" s="42" t="n">
+        <v>29.32450416163935</v>
+      </c>
+      <c r="D5" s="42" t="n">
+        <v>22.50669926600663</v>
+      </c>
+      <c r="E5" s="42" t="n">
+        <v>65.79207921795091</v>
+      </c>
+      <c r="F5" s="42" t="n">
+        <v>158.4741112911011</v>
+      </c>
+      <c r="G5" s="42" t="n">
+        <v>155.0819687122736</v>
+      </c>
+      <c r="H5" s="42" t="n">
+        <v>261.3663162682093</v>
+      </c>
+      <c r="I5" s="42" t="n">
+        <v>253.4120620304224</v>
+      </c>
+      <c r="J5" s="42" t="n">
+        <v>434.0875008000365</v>
+      </c>
+      <c r="K5" s="42" t="n">
+        <v>253.5475481809133</v>
+      </c>
+      <c r="L5" s="42" t="n">
+        <v>302.7226418468389</v>
+      </c>
+      <c r="M5" s="42" t="n">
+        <v>393.0673276715649</v>
+      </c>
+      <c r="N5" s="42" t="n">
+        <v>768.9158122024958</v>
+      </c>
+      <c r="O5" s="42" t="n">
+        <v>2405.752892732271</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="n">
+        <v>-3.555866059064835</v>
+      </c>
+      <c r="C6" s="42" t="n">
+        <v>-111.7459765360536</v>
+      </c>
+      <c r="D6" s="42" t="n">
+        <v>-110.466314823209</v>
+      </c>
+      <c r="E6" s="42" t="n">
+        <v>-95.51521086948183</v>
+      </c>
+      <c r="F6" s="42" t="n">
+        <v>-169.7874453691625</v>
+      </c>
+      <c r="G6" s="42" t="n">
+        <v>-282.6790926905302</v>
+      </c>
+      <c r="H6" s="42" t="n">
+        <v>-1.788139343261719e-13</v>
+      </c>
+      <c r="I6" s="42" t="n">
+        <v>178.254073047358</v>
+      </c>
+      <c r="J6" s="42" t="n">
+        <v>364.5072857408031</v>
+      </c>
+      <c r="K6" s="42" t="n">
+        <v>251.5494596101897</v>
+      </c>
+      <c r="L6" s="42" t="n">
+        <v>249.4154198916363</v>
+      </c>
+      <c r="M6" s="42" t="n">
+        <v>318.4954012590323</v>
+      </c>
+      <c r="N6" s="42" t="n">
+        <v>-773.7499063475022</v>
+      </c>
+      <c r="O6" s="42" t="n">
+        <v>588.4717332015173</v>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>Total OPEX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="n">
+        <v>-125.34267815</v>
+      </c>
+      <c r="C9" s="42" t="n">
+        <v>-99.25214621000001</v>
+      </c>
+      <c r="D9" s="42" t="n">
+        <v>-86.70986521020025</v>
+      </c>
+      <c r="E9" s="42" t="n">
+        <v>-193.3246613008188</v>
+      </c>
+      <c r="F9" s="42" t="n">
+        <v>-160.1465483796875</v>
+      </c>
+      <c r="G9" s="42" t="n">
+        <v>-243.8601949635304</v>
+      </c>
+      <c r="H9" s="42" t="n">
+        <v>-224.8392573646601</v>
+      </c>
+      <c r="I9" s="42" t="n">
+        <v>-125.0265121653656</v>
+      </c>
+      <c r="J9" s="42" t="n">
+        <v>-188.242606259593</v>
+      </c>
+      <c r="K9" s="42" t="n">
+        <v>-157.3424379705963</v>
+      </c>
+      <c r="L9" s="42" t="n">
+        <v>-179.2331266195248</v>
+      </c>
+      <c r="M9" s="42" t="n">
+        <v>-252.9619797635129</v>
+      </c>
+      <c r="N9" s="42" t="n">
+        <v>-1133.475351578897</v>
+      </c>
+      <c r="O9" s="42" t="n">
+        <v>-2036.28201435749</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="n">
+        <v>-125.3387091217621</v>
+      </c>
+      <c r="C10" s="42" t="n">
+        <v>-114.3157810228943</v>
+      </c>
+      <c r="D10" s="42" t="n">
+        <v>-124.3046163602002</v>
+      </c>
+      <c r="E10" s="42" t="n">
+        <v>-141.6458343208189</v>
+      </c>
+      <c r="F10" s="42" t="n">
+        <v>-158.9793936550312</v>
+      </c>
+      <c r="G10" s="42" t="n">
+        <v>-231.4114917358956</v>
+      </c>
+      <c r="H10" s="42" t="n">
+        <v>-237.2664831622952</v>
+      </c>
+      <c r="I10" s="42" t="n">
+        <v>-204.575265598262</v>
+      </c>
+      <c r="J10" s="42" t="n">
+        <v>-73.68972297248567</v>
+      </c>
+      <c r="K10" s="42" t="n">
+        <v>-226.8061106085225</v>
+      </c>
+      <c r="L10" s="42" t="n">
+        <v>-220.8601433316447</v>
+      </c>
+      <c r="M10" s="42" t="n">
+        <v>-235.6814881808957</v>
+      </c>
+      <c r="N10" s="42" t="n">
+        <v>-1133.262309378897</v>
+      </c>
+      <c r="O10" s="42" t="n">
+        <v>-2094.875040070708</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="n">
+        <v>0.003969028237938881</v>
+      </c>
+      <c r="C11" s="42" t="n">
+        <v>-15.06363481289428</v>
+      </c>
+      <c r="D11" s="42" t="n">
+        <v>-37.59475114999998</v>
+      </c>
+      <c r="E11" s="42" t="n">
+        <v>51.6788269799999</v>
+      </c>
+      <c r="F11" s="42" t="n">
+        <v>1.167154724656284</v>
+      </c>
+      <c r="G11" s="42" t="n">
+        <v>12.44870322763479</v>
+      </c>
+      <c r="H11" s="42" t="n">
+        <v>-12.42722579763508</v>
+      </c>
+      <c r="I11" s="42" t="n">
+        <v>-79.54875343289646</v>
+      </c>
+      <c r="J11" s="42" t="n">
+        <v>114.5528832871074</v>
+      </c>
+      <c r="K11" s="42" t="n">
+        <v>-69.46367263792622</v>
+      </c>
+      <c r="L11" s="42" t="n">
+        <v>-41.62701671211982</v>
+      </c>
+      <c r="M11" s="42" t="n">
+        <v>17.28049158261719</v>
+      </c>
+      <c r="N11" s="42" t="n">
+        <v>0.2130421999995665</v>
+      </c>
+      <c r="O11" s="42" t="n">
+        <v>-58.59302571321837</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>PEX admin</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="n">
+        <v>-92.88636049999999</v>
+      </c>
+      <c r="C14" s="42" t="n">
+        <v>-94.5925139</v>
+      </c>
+      <c r="D14" s="42" t="n">
+        <v>-95.10917844724878</v>
+      </c>
+      <c r="E14" s="42" t="n">
+        <v>-101.8822365107256</v>
+      </c>
+      <c r="F14" s="42" t="n">
+        <v>-112.4676209260646</v>
+      </c>
+      <c r="G14" s="42" t="n">
+        <v>-106.2402667461649</v>
+      </c>
+      <c r="H14" s="42" t="n">
+        <v>-101.3368353946933</v>
+      </c>
+      <c r="I14" s="42" t="n">
+        <v>-93.65857750675626</v>
+      </c>
+      <c r="J14" s="42" t="n">
+        <v>-99.31385958187134</v>
+      </c>
+      <c r="K14" s="42" t="n">
+        <v>-104.4993205606332</v>
+      </c>
+      <c r="L14" s="42" t="n">
+        <v>-105.0015625884656</v>
+      </c>
+      <c r="M14" s="42" t="n">
+        <v>-106.5198882024433</v>
+      </c>
+      <c r="N14" s="42" t="n">
+        <v>-704.5150124248971</v>
+      </c>
+      <c r="O14" s="42" t="n">
+        <v>-1213.508220865067</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="n">
+        <v>-89.79414117176206</v>
+      </c>
+      <c r="C15" s="42" t="n">
+        <v>-91.05581404346746</v>
+      </c>
+      <c r="D15" s="42" t="n">
+        <v>-91.79054847724878</v>
+      </c>
+      <c r="E15" s="42" t="n">
+        <v>-102.5217923807257</v>
+      </c>
+      <c r="F15" s="42" t="n">
+        <v>-106.1266098708351</v>
+      </c>
+      <c r="G15" s="42" t="n">
+        <v>-109.2490030885301</v>
+      </c>
+      <c r="H15" s="42" t="n">
+        <v>-113.9771033923283</v>
+      </c>
+      <c r="I15" s="42" t="n">
+        <v>-111.3047417725611</v>
+      </c>
+      <c r="J15" s="42" t="n">
+        <v>44.82120126104592</v>
+      </c>
+      <c r="K15" s="42" t="n">
+        <v>-111.5102827511398</v>
+      </c>
+      <c r="L15" s="42" t="n">
+        <v>-111.5102827511398</v>
+      </c>
+      <c r="M15" s="42" t="n">
+        <v>-111.5102827511398</v>
+      </c>
+      <c r="N15" s="42" t="n">
+        <v>-704.5150124248976</v>
+      </c>
+      <c r="O15" s="42" t="n">
+        <v>-1105.529401189832</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="n">
+        <v>3.092219328237936</v>
+      </c>
+      <c r="C16" s="42" t="n">
+        <v>3.536699856532544</v>
+      </c>
+      <c r="D16" s="42" t="n">
+        <v>3.318629970000014</v>
+      </c>
+      <c r="E16" s="42" t="n">
+        <v>-0.6395558700000793</v>
+      </c>
+      <c r="F16" s="42" t="n">
+        <v>6.341011055229485</v>
+      </c>
+      <c r="G16" s="42" t="n">
+        <v>-3.00873634236525</v>
+      </c>
+      <c r="H16" s="42" t="n">
+        <v>-12.6402679976351</v>
+      </c>
+      <c r="I16" s="42" t="n">
+        <v>-17.64616426580484</v>
+      </c>
+      <c r="J16" s="42" t="n">
+        <v>144.1350608429173</v>
+      </c>
+      <c r="K16" s="42" t="n">
+        <v>-7.010962190506592</v>
+      </c>
+      <c r="L16" s="42" t="n">
+        <v>-6.508720162674174</v>
+      </c>
+      <c r="M16" s="42" t="n">
+        <v>-4.990394548696548</v>
+      </c>
+      <c r="N16" s="42" t="n">
+        <v>-4.464206782017754e-13</v>
+      </c>
+      <c r="O16" s="42" t="n">
+        <v>107.9788196752346</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>PEX other</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="n">
+        <v>-3.05173</v>
+      </c>
+      <c r="C19" s="42" t="n">
+        <v>-0.442289</v>
+      </c>
+      <c r="D19" s="42" t="n">
+        <v>-1.224642702951454</v>
+      </c>
+      <c r="E19" s="42" t="n">
+        <v>-1.641531440093187</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <v>-1.239698623622975</v>
+      </c>
+      <c r="G19" s="42" t="n">
+        <v>-16.41692346736547</v>
+      </c>
+      <c r="H19" s="42" t="n">
+        <v>2.264459930033199</v>
+      </c>
+      <c r="I19" s="42" t="n">
+        <v>16.7480517006507</v>
+      </c>
+      <c r="J19" s="42" t="n">
+        <v>2.180891466245528</v>
+      </c>
+      <c r="K19" s="42" t="n">
+        <v>-5.028727824454847</v>
+      </c>
+      <c r="L19" s="42" t="n">
+        <v>-6.046734866731608</v>
+      </c>
+      <c r="M19" s="42" t="n">
+        <v>-8.404824671504404</v>
+      </c>
+      <c r="N19" s="42" t="n">
+        <v>-21.75235530399989</v>
+      </c>
+      <c r="O19" s="42" t="n">
+        <v>-22.30369949979452</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="n">
+        <v>-6.095354879999999</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>-3.930295659426838</v>
+      </c>
+      <c r="D20" s="42" t="n">
+        <v>-4.512458402951454</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>-0.968213230093187</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>-6.764981754196137</v>
+      </c>
+      <c r="G20" s="42" t="n">
+        <v>-1.745511307365466</v>
+      </c>
+      <c r="H20" s="42" t="n">
+        <v>2.2644599300332</v>
+      </c>
+      <c r="I20" s="42" t="n">
+        <v>-3.169988265700941</v>
+      </c>
+      <c r="J20" s="42" t="n">
+        <v>-0.4110462535315826</v>
+      </c>
+      <c r="K20" s="42" t="n">
+        <v>-4.272655524947914</v>
+      </c>
+      <c r="L20" s="42" t="n">
+        <v>-4.142931662061526</v>
+      </c>
+      <c r="M20" s="42" t="n">
+        <v>-3.965340224999997</v>
+      </c>
+      <c r="N20" s="42" t="n">
+        <v>-21.75235530399988</v>
+      </c>
+      <c r="O20" s="42" t="n">
+        <v>-37.71431723524184</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="n">
+        <v>-3.04362488</v>
+      </c>
+      <c r="C21" s="42" t="n">
+        <v>-3.488006659426838</v>
+      </c>
+      <c r="D21" s="42" t="n">
+        <v>-3.2878157</v>
+      </c>
+      <c r="E21" s="42" t="n">
+        <v>0.67331821</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <v>-5.525283130573162</v>
+      </c>
+      <c r="G21" s="42" t="n">
+        <v>14.67141216</v>
+      </c>
+      <c r="H21" s="42" t="n">
+        <v>9.313225746154785e-16</v>
+      </c>
+      <c r="I21" s="42" t="n">
+        <v>-19.91803996635164</v>
+      </c>
+      <c r="J21" s="42" t="n">
+        <v>-2.591937719777111</v>
+      </c>
+      <c r="K21" s="42" t="n">
+        <v>0.7560722995069324</v>
+      </c>
+      <c r="L21" s="42" t="n">
+        <v>1.903803204670082</v>
+      </c>
+      <c r="M21" s="42" t="n">
+        <v>4.439484446504408</v>
+      </c>
+      <c r="N21" s="42" t="n">
+        <v>5.261192370653589e-15</v>
+      </c>
+      <c r="O21" s="42" t="n">
+        <v>-15.41061773544732</v>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="n">
+        <v>-28.528894</v>
+      </c>
+      <c r="C24" s="42" t="n">
+        <v>-1.745</v>
+      </c>
+      <c r="D24" s="42" t="n">
+        <v>9.53520363</v>
+      </c>
+      <c r="E24" s="42" t="n">
+        <v>-87.75989982000003</v>
+      </c>
+      <c r="F24" s="42" t="n">
+        <v>-43.87168396999997</v>
+      </c>
+      <c r="G24" s="42" t="n">
+        <v>-106.62055019</v>
+      </c>
+      <c r="H24" s="42" t="n">
+        <v>-120.26675859</v>
+      </c>
+      <c r="I24" s="42" t="n">
+        <v>-36.70756957093808</v>
+      </c>
+      <c r="J24" s="42" t="n">
+        <v>-78.88946415094287</v>
+      </c>
+      <c r="K24" s="42" t="n">
+        <v>-35.09308791370314</v>
+      </c>
+      <c r="L24" s="42" t="n">
+        <v>-53.47374275074998</v>
+      </c>
+      <c r="M24" s="42" t="n">
+        <v>-103.7866509770251</v>
+      </c>
+      <c r="N24" s="42" t="n">
+        <v>-379.2575829400001</v>
+      </c>
+      <c r="O24" s="42" t="n">
+        <v>-687.2080983033592</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="n">
+        <v>-28.52889409</v>
+      </c>
+      <c r="C25" s="42" t="n">
+        <v>-16.82913428</v>
+      </c>
+      <c r="D25" s="42" t="n">
+        <v>-27.05948898</v>
+      </c>
+      <c r="E25" s="42" t="n">
+        <v>-36.08107284000001</v>
+      </c>
+      <c r="F25" s="42" t="n">
+        <v>-43.76846497</v>
+      </c>
+      <c r="G25" s="42" t="n">
+        <v>-106.72376919</v>
+      </c>
+      <c r="H25" s="42" t="n">
+        <v>-120.26579917</v>
+      </c>
+      <c r="I25" s="42" t="n">
+        <v>-82.79719141</v>
+      </c>
+      <c r="J25" s="42" t="n">
+        <v>-105.089188</v>
+      </c>
+      <c r="K25" s="42" t="n">
+        <v>-104.6528311930226</v>
+      </c>
+      <c r="L25" s="42" t="n">
+        <v>-98.20793697621149</v>
+      </c>
+      <c r="M25" s="42" t="n">
+        <v>-111.6228575142901</v>
+      </c>
+      <c r="N25" s="42" t="n">
+        <v>-379.2566235200001</v>
+      </c>
+      <c r="O25" s="42" t="n">
+        <v>-881.6266286135242</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B26" s="42" t="n">
+        <v>-8.999999985098839e-08</v>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>-15.08413428</v>
+      </c>
+      <c r="D26" s="42" t="n">
+        <v>-36.59469261</v>
+      </c>
+      <c r="E26" s="42" t="n">
+        <v>51.67882698000001</v>
+      </c>
+      <c r="F26" s="42" t="n">
+        <v>0.1032189999999702</v>
+      </c>
+      <c r="G26" s="42" t="n">
+        <v>-0.1032189999999851</v>
+      </c>
+      <c r="H26" s="42" t="n">
+        <v>0.0009594200000017882</v>
+      </c>
+      <c r="I26" s="42" t="n">
+        <v>-46.08962183906191</v>
+      </c>
+      <c r="J26" s="42" t="n">
+        <v>-26.19972384905712</v>
+      </c>
+      <c r="K26" s="42" t="n">
+        <v>-69.55974327931945</v>
+      </c>
+      <c r="L26" s="42" t="n">
+        <v>-44.73419422546151</v>
+      </c>
+      <c r="M26" s="42" t="n">
+        <v>-7.836206537265018</v>
+      </c>
+      <c r="N26" s="42" t="n">
+        <v>0.000959419999994479</v>
+      </c>
+      <c r="O26" s="42" t="n">
+        <v>-194.418530310165</v>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>Consulting and insurance</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="n">
+        <v>-0.155854</v>
+      </c>
+      <c r="C29" s="42" t="n">
+        <v>-1.633817</v>
+      </c>
+      <c r="D29" s="42" t="n">
+        <v>0.77247476</v>
+      </c>
+      <c r="E29" s="42" t="n">
+        <v>-1.37120632</v>
+      </c>
+      <c r="F29" s="42" t="n">
+        <v>-2.464153540000001</v>
+      </c>
+      <c r="G29" s="42" t="n">
+        <v>-2.164074739999998</v>
+      </c>
+      <c r="H29" s="42" t="n">
+        <v>-0.9401674499999998</v>
+      </c>
+      <c r="I29" s="42" t="n">
+        <v>-4.51437680711905</v>
+      </c>
+      <c r="J29" s="42" t="n">
+        <v>-4.51437680711905</v>
+      </c>
+      <c r="K29" s="42" t="n">
+        <v>-4.20437680711905</v>
+      </c>
+      <c r="L29" s="42" t="n">
+        <v>-4.20437680711905</v>
+      </c>
+      <c r="M29" s="42" t="n">
+        <v>-4.23437680711905</v>
+      </c>
+      <c r="N29" s="42" t="n">
+        <v>-7.956798289999999</v>
+      </c>
+      <c r="O29" s="42" t="n">
+        <v>-29.62868232559525</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="n">
+        <v>-0.15585397</v>
+      </c>
+      <c r="C30" s="42" t="n">
+        <v>-1.63381665</v>
+      </c>
+      <c r="D30" s="42" t="n">
+        <v>-0.20311578</v>
+      </c>
+      <c r="E30" s="42" t="n">
+        <v>-1.37120632</v>
+      </c>
+      <c r="F30" s="42" t="n">
+        <v>-1.48856338</v>
+      </c>
+      <c r="G30" s="42" t="n">
+        <v>-2.16407474</v>
+      </c>
+      <c r="H30" s="42" t="n">
+        <v>-0.7221537499999998</v>
+      </c>
+      <c r="I30" s="42" t="n">
+        <v>-0.96429323</v>
+      </c>
+      <c r="J30" s="42" t="n">
+        <v>-3.887514700000001</v>
+      </c>
+      <c r="K30" s="42" t="n">
+        <v>-1.28350724</v>
+      </c>
+      <c r="L30" s="42" t="n">
+        <v>-1.28350724</v>
+      </c>
+      <c r="M30" s="42" t="n">
+        <v>-1.28350724</v>
+      </c>
+      <c r="N30" s="42" t="n">
+        <v>-7.73878459</v>
+      </c>
+      <c r="O30" s="42" t="n">
+        <v>-16.44111424</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B31" s="42" t="n">
+        <v>2.999999999883585e-08</v>
+      </c>
+      <c r="C31" s="42" t="n">
+        <v>3.499999998603016e-07</v>
+      </c>
+      <c r="D31" s="42" t="n">
+        <v>-0.97559054</v>
+      </c>
+      <c r="E31" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="42" t="n">
+        <v>0.9755901600000011</v>
+      </c>
+      <c r="G31" s="42" t="n">
+        <v>-1.862645149230957e-15</v>
+      </c>
+      <c r="H31" s="42" t="n">
+        <v>0.2180137000000001</v>
+      </c>
+      <c r="I31" s="42" t="n">
+        <v>3.55008357711905</v>
+      </c>
+      <c r="J31" s="42" t="n">
+        <v>0.6268621071190494</v>
+      </c>
+      <c r="K31" s="42" t="n">
+        <v>2.92086956711905</v>
+      </c>
+      <c r="L31" s="42" t="n">
+        <v>2.92086956711905</v>
+      </c>
+      <c r="M31" s="42" t="n">
+        <v>2.95086956711905</v>
+      </c>
+      <c r="N31" s="42" t="n">
+        <v>0.2180136999999991</v>
+      </c>
+      <c r="O31" s="42" t="n">
+        <v>13.18756808559525</v>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="41" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="n">
+        <v>-0.7198396500000001</v>
+      </c>
+      <c r="C34" s="42" t="n">
+        <v>-0.8385263100000001</v>
+      </c>
+      <c r="D34" s="42" t="n">
+        <v>-0.6837224500000001</v>
+      </c>
+      <c r="E34" s="42" t="n">
+        <v>-0.6697872100000001</v>
+      </c>
+      <c r="F34" s="42" t="n">
+        <v>-0.1033913200000003</v>
+      </c>
+      <c r="G34" s="42" t="n">
+        <v>-12.41837982</v>
+      </c>
+      <c r="H34" s="42" t="n">
+        <v>-4.55995586</v>
+      </c>
+      <c r="I34" s="42" t="n">
+        <v>-6.894039981202883</v>
+      </c>
+      <c r="J34" s="42" t="n">
+        <v>-7.70579718590529</v>
+      </c>
+      <c r="K34" s="42" t="n">
+        <v>-8.516924864686031</v>
+      </c>
+      <c r="L34" s="42" t="n">
+        <v>-10.50670960645853</v>
+      </c>
+      <c r="M34" s="42" t="n">
+        <v>-30.01623910542114</v>
+      </c>
+      <c r="N34" s="42" t="n">
+        <v>-19.99360262</v>
+      </c>
+      <c r="O34" s="42" t="n">
+        <v>-83.63331336367386</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B35" s="42" t="n">
+        <v>-0.7644650100000001</v>
+      </c>
+      <c r="C35" s="42" t="n">
+        <v>-0.86672039</v>
+      </c>
+      <c r="D35" s="42" t="n">
+        <v>-0.7390047199999999</v>
+      </c>
+      <c r="E35" s="42" t="n">
+        <v>-0.7035495500000001</v>
+      </c>
+      <c r="F35" s="42" t="n">
+        <v>-0.83077368</v>
+      </c>
+      <c r="G35" s="42" t="n">
+        <v>-11.52913341</v>
+      </c>
+      <c r="H35" s="42" t="n">
+        <v>-4.56588678</v>
+      </c>
+      <c r="I35" s="42" t="n">
+        <v>-6.339050920000001</v>
+      </c>
+      <c r="J35" s="42" t="n">
+        <v>-9.12317528</v>
+      </c>
+      <c r="K35" s="42" t="n">
+        <v>-5.086833899412203</v>
+      </c>
+      <c r="L35" s="42" t="n">
+        <v>-5.71548470223184</v>
+      </c>
+      <c r="M35" s="42" t="n">
+        <v>-7.299500450465856</v>
+      </c>
+      <c r="N35" s="42" t="n">
+        <v>-19.99953354</v>
+      </c>
+      <c r="O35" s="42" t="n">
+        <v>-53.5635787921099</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B36" s="42" t="n">
+        <v>-0.0446253600000001</v>
+      </c>
+      <c r="C36" s="42" t="n">
+        <v>-0.02819407999999996</v>
+      </c>
+      <c r="D36" s="42" t="n">
+        <v>-0.0552822699999999</v>
+      </c>
+      <c r="E36" s="42" t="n">
+        <v>-0.03376233999999997</v>
+      </c>
+      <c r="F36" s="42" t="n">
+        <v>-0.7273823599999997</v>
+      </c>
+      <c r="G36" s="42" t="n">
+        <v>0.8892464100000002</v>
+      </c>
+      <c r="H36" s="42" t="n">
+        <v>-0.005930919999999926</v>
+      </c>
+      <c r="I36" s="42" t="n">
+        <v>0.5549890612028818</v>
+      </c>
+      <c r="J36" s="42" t="n">
+        <v>-1.417378094094709</v>
+      </c>
+      <c r="K36" s="42" t="n">
+        <v>3.430090965273828</v>
+      </c>
+      <c r="L36" s="42" t="n">
+        <v>4.79122490422669</v>
+      </c>
+      <c r="M36" s="42" t="n">
+        <v>22.71673865495528</v>
+      </c>
+      <c r="N36" s="42" t="n">
+        <v>-0.005930919999999374</v>
+      </c>
+      <c r="O36" s="42" t="n">
+        <v>30.06973457156397</v>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Янв–Июл</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  было</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="n">
+        <v>-45.41667880562037</v>
+      </c>
+      <c r="C39" s="42" t="n">
+        <v>41.81833448769292</v>
+      </c>
+      <c r="D39" s="42" t="n">
+        <v>46.26314887901543</v>
+      </c>
+      <c r="E39" s="42" t="n">
+        <v>-32.01737121338606</v>
+      </c>
+      <c r="F39" s="42" t="n">
+        <v>168.1150082805762</v>
+      </c>
+      <c r="G39" s="42" t="n">
+        <v>193.9008664392734</v>
+      </c>
+      <c r="H39" s="42" t="n">
+        <v>36.52705890354943</v>
+      </c>
+      <c r="I39" s="42" t="n">
+        <v>-49.86852318230127</v>
+      </c>
+      <c r="J39" s="42" t="n">
+        <v>-118.6623912003597</v>
+      </c>
+      <c r="K39" s="42" t="n">
+        <v>-155.3443493998727</v>
+      </c>
+      <c r="L39" s="42" t="n">
+        <v>-125.9259046643223</v>
+      </c>
+      <c r="M39" s="42" t="n">
+        <v>-178.3900533509803</v>
+      </c>
+      <c r="N39" s="42" t="n">
+        <v>409.1903669711009</v>
+      </c>
+      <c r="O39" s="42" t="n">
+        <v>-219.0008548267354</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  стало</t>
+        </is>
+      </c>
+      <c r="B40" s="42" t="n">
+        <v>-48.96857583644727</v>
+      </c>
+      <c r="C40" s="42" t="n">
+        <v>-84.99127686125495</v>
+      </c>
+      <c r="D40" s="42" t="n">
+        <v>-101.7979170941936</v>
+      </c>
+      <c r="E40" s="42" t="n">
+        <v>-75.85375510286799</v>
+      </c>
+      <c r="F40" s="42" t="n">
+        <v>-0.5052823639300763</v>
+      </c>
+      <c r="G40" s="42" t="n">
+        <v>-76.32952302362203</v>
+      </c>
+      <c r="H40" s="42" t="n">
+        <v>24.09983310591418</v>
+      </c>
+      <c r="I40" s="42" t="n">
+        <v>48.83679643216032</v>
+      </c>
+      <c r="J40" s="42" t="n">
+        <v>360.3977778275508</v>
+      </c>
+      <c r="K40" s="42" t="n">
+        <v>26.74143757239073</v>
+      </c>
+      <c r="L40" s="42" t="n">
+        <v>81.86249851519423</v>
+      </c>
+      <c r="M40" s="42" t="n">
+        <v>157.3858394906691</v>
+      </c>
+      <c r="N40" s="42" t="n">
+        <v>-364.3464971764017</v>
+      </c>
+      <c r="O40" s="42" t="n">
+        <v>310.8778526615635</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ</t>
+        </is>
+      </c>
+      <c r="B41" s="42" t="n">
+        <v>-3.551897030826896</v>
+      </c>
+      <c r="C41" s="42" t="n">
+        <v>-126.8096113489479</v>
+      </c>
+      <c r="D41" s="42" t="n">
+        <v>-148.061065973209</v>
+      </c>
+      <c r="E41" s="42" t="n">
+        <v>-43.83638388948193</v>
+      </c>
+      <c r="F41" s="42" t="n">
+        <v>-168.6202906445062</v>
+      </c>
+      <c r="G41" s="42" t="n">
+        <v>-270.2303894628954</v>
+      </c>
+      <c r="H41" s="42" t="n">
+        <v>-12.42722579763526</v>
+      </c>
+      <c r="I41" s="42" t="n">
+        <v>98.70531961446159</v>
+      </c>
+      <c r="J41" s="42" t="n">
+        <v>479.0601690279105</v>
+      </c>
+      <c r="K41" s="42" t="n">
+        <v>182.0857869722635</v>
+      </c>
+      <c r="L41" s="42" t="n">
+        <v>207.7884031795165</v>
+      </c>
+      <c r="M41" s="42" t="n">
+        <v>335.7758928416495</v>
+      </c>
+      <c r="N41" s="42" t="n">
+        <v>-773.5368641475026</v>
+      </c>
+      <c r="O41" s="42" t="n">
+        <v>529.878707488299</v>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Логика нового свода:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Commercial margin = инкремент без E-comm по контрагентам (4 правила, BiP, без ADJ: 12 Сегменты стр. 13+15) + вознаграждения РА и блогерам (10 PL стр. 17+18) — так собран июль в прежнем своде (FC Summary стр. 15 авг. мастера).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OPEX — значения месяца из 10 PL мастера (факт / предфакт сентября / прогноз окт–дек).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Прежний свод янв–июн: янв–апр вбиты из старых версий, май–июн — накопленный итог по инкременту С E-comm (ЗФ стр. 101) минус прошлые месяцы; OPEX — значения на дату закрытия.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
October forecast: revenue -7/31 for app outage (summary, E-Com, deck); master unchanged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142u1JgEJ5Z4iqbgjpLWfcB
</commit_message>
<xml_diff>
--- a/Adtech_svod_Aug-Sep_fact_Oct-Dec_FC.xlsx
+++ b/Adtech_svod_Aug-Sep_fact_Oct-Dec_FC.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:N64"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="51.83203125" customWidth="1" min="1" max="1"/>
@@ -709,6 +709,13 @@
     <col width="11.1640625" customWidth="1" style="35" min="14" max="14"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>окт: выручка −7/31 (сбой приложения), −65.8 млн</t>
+        </is>
+      </c>
+    </row>
     <row r="2" ht="16" customHeight="1" thickBot="1">
       <c r="B2" s="38" t="inlineStr">
         <is>
@@ -1113,7 +1120,7 @@
         <v>434087500.8000364</v>
       </c>
       <c r="K16" s="18" t="n">
-        <v>253547548.1809133</v>
+        <v>187706013.2808443</v>
       </c>
       <c r="L16" s="18" t="n">
         <v>302722641.8468388</v>
@@ -1337,7 +1344,7 @@
         <v>434087500.8000364</v>
       </c>
       <c r="K26" s="24" t="n">
-        <v>253547548.1809133</v>
+        <v>187706013.2808443</v>
       </c>
       <c r="L26" s="24" t="n">
         <v>302722641.8468388</v>
@@ -2233,7 +2240,7 @@
         <v>360397777.8275508</v>
       </c>
       <c r="K60" s="24" t="n">
-        <v>26741437.57239074</v>
+        <v>-39100097.32767828</v>
       </c>
       <c r="L60" s="24" t="n">
         <v>81862498.51519418</v>

</xml_diff>